<commit_message>
Update signal logs, token cache, and service files
</commit_message>
<xml_diff>
--- a/Mine/signal_logs_highlow.xlsx
+++ b/Mine/signal_logs_highlow.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2387,6 +2387,1938 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:20:00</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>09:20:00</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:25:00</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>09:25:00</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:30:00</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:35:00</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:40:00</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>09:40:00</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:45:00</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>09:45:00</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr"/>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:50:00</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>09:50:00</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 09:55:00</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>09:55:00</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr"/>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:20:00</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>10:20:00</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:25:00</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>10:25:00</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:30:00</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:35:00</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>10:35:00</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:40:00</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>10:40:00</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:45:00</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>10:45:00</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:50:00</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>10:50:00</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 10:55:00</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>10:55:00</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:20:00</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:25:00</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>11:25:00</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:30:00</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:35:00</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:40:00</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>11:40:00</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:45:00</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr"/>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:50:00</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>11:50:00</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr"/>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 11:55:00</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>11:55:00</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr"/>
+      <c r="N69" s="2" t="inlineStr"/>
+      <c r="O69" s="2" t="inlineStr"/>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:20:00</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>12:20:00</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr"/>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:25:00</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr"/>
+      <c r="N71" s="2" t="inlineStr"/>
+      <c r="O71" s="2" t="inlineStr"/>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:30:00</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr"/>
+      <c r="N72" s="2" t="inlineStr"/>
+      <c r="O72" s="2" t="inlineStr"/>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:35:00</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>12:35:00</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr"/>
+      <c r="N73" s="2" t="inlineStr"/>
+      <c r="O73" s="2" t="inlineStr"/>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:40:00</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>12:40:00</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:45:00</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr"/>
+      <c r="N75" s="2" t="inlineStr"/>
+      <c r="O75" s="2" t="inlineStr"/>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:50:00</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr"/>
+      <c r="O76" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:55:00</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>12:55:00</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr"/>
+      <c r="O77" s="2" t="inlineStr"/>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:35:37</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>13:35:37</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr"/>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:49:16</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>13:49:16</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr"/>
+      <c r="N79" s="2" t="inlineStr"/>
+      <c r="O79" s="2" t="inlineStr"/>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:49:17</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>13:49:17</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr"/>
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:50:00</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr"/>
+      <c r="N81" s="2" t="inlineStr"/>
+      <c r="O81" s="2" t="inlineStr"/>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:55:00</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="inlineStr"/>
+      <c r="O82" s="2" t="inlineStr"/>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:20:00</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="inlineStr"/>
+      <c r="O83" s="2" t="inlineStr"/>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:25:00</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:30:00</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="inlineStr"/>
+      <c r="O85" s="2" t="inlineStr"/>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:35:00</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr"/>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:40:00</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr"/>
+      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr"/>
+      <c r="N87" s="2" t="inlineStr"/>
+      <c r="O87" s="2" t="inlineStr"/>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:45:00</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr"/>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:50:00</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr"/>
+      <c r="O89" s="2" t="inlineStr"/>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 14:55:00</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr"/>
+      <c r="O90" s="2" t="inlineStr"/>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 15:20:00</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>15:20:00</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr"/>
+      <c r="N91" s="2" t="inlineStr"/>
+      <c r="O91" s="2" t="inlineStr"/>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: remove temporary Excel file lock
</commit_message>
<xml_diff>
--- a/Mine/signal_logs_highlow.xlsx
+++ b/Mine/signal_logs_highlow.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:P140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4319,6 +4319,2064 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:20:00</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>09:20:00</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr"/>
+      <c r="N92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr"/>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:25:00</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>09:25:00</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr"/>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr"/>
+      <c r="O93" s="2" t="inlineStr"/>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:30:00</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr"/>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:35:00</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>09:35:00</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr"/>
+      <c r="O95" s="2" t="inlineStr"/>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:40:00</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>09:40:00</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr"/>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:46:44</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>09:46:44</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>09:46</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr"/>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr"/>
+      <c r="O97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:50:00</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>09:50:00</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr"/>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 09:55:00</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>09:55:00</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr"/>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr"/>
+      <c r="N99" s="2" t="inlineStr"/>
+      <c r="O99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:20:01</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>10:20:01</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr"/>
+      <c r="O100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:25:00</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>10:25:00</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr"/>
+      <c r="N101" s="2" t="inlineStr"/>
+      <c r="O101" s="2" t="inlineStr"/>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:30:00</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr"/>
+      <c r="E102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr"/>
+      <c r="M102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr"/>
+      <c r="O102" s="2" t="inlineStr"/>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:35:00</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>10:35:00</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr"/>
+      <c r="E103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr"/>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr"/>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr"/>
+      <c r="M103" s="2" t="inlineStr"/>
+      <c r="N103" s="2" t="inlineStr"/>
+      <c r="O103" s="2" t="inlineStr"/>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:40:00</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>10:40:00</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr"/>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:45:00</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>10:45:00</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr"/>
+      <c r="E105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr"/>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr"/>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr"/>
+      <c r="M105" s="2" t="inlineStr"/>
+      <c r="N105" s="2" t="inlineStr"/>
+      <c r="O105" s="2" t="inlineStr"/>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:50:00</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>10:50:00</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr"/>
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr"/>
+      <c r="M106" s="2" t="inlineStr"/>
+      <c r="N106" s="2" t="inlineStr"/>
+      <c r="O106" s="2" t="inlineStr"/>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 10:55:00</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>10:55:00</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr"/>
+      <c r="E107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr"/>
+      <c r="G107" s="2" t="inlineStr"/>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr"/>
+      <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr"/>
+      <c r="M107" s="2" t="inlineStr"/>
+      <c r="N107" s="2" t="inlineStr"/>
+      <c r="O107" s="2" t="inlineStr"/>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:20:00</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr"/>
+      <c r="E108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr"/>
+      <c r="G108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
+      <c r="L108" s="2" t="inlineStr"/>
+      <c r="M108" s="2" t="inlineStr"/>
+      <c r="N108" s="2" t="inlineStr"/>
+      <c r="O108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:25:01</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>11:25:01</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr"/>
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="2" t="inlineStr"/>
+      <c r="M109" s="2" t="inlineStr"/>
+      <c r="N109" s="2" t="inlineStr"/>
+      <c r="O109" s="2" t="inlineStr"/>
+      <c r="P109" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:30:00</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>11:30:00</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr"/>
+      <c r="G110" s="2" t="inlineStr"/>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr"/>
+      <c r="M110" s="2" t="inlineStr"/>
+      <c r="N110" s="2" t="inlineStr"/>
+      <c r="O110" s="2" t="inlineStr"/>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:35:00</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr"/>
+      <c r="G111" s="2" t="inlineStr"/>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr"/>
+      <c r="K111" s="2" t="inlineStr"/>
+      <c r="L111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr"/>
+      <c r="N111" s="2" t="inlineStr"/>
+      <c r="O111" s="2" t="inlineStr"/>
+      <c r="P111" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:40:00</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>11:40:00</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr"/>
+      <c r="E112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr"/>
+      <c r="G112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr"/>
+      <c r="M112" s="2" t="inlineStr"/>
+      <c r="N112" s="2" t="inlineStr"/>
+      <c r="O112" s="2" t="inlineStr"/>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:45:00</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>11:45:00</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr"/>
+      <c r="E113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr"/>
+      <c r="G113" s="2" t="inlineStr"/>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr"/>
+      <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="2" t="inlineStr"/>
+      <c r="M113" s="2" t="inlineStr"/>
+      <c r="N113" s="2" t="inlineStr"/>
+      <c r="O113" s="2" t="inlineStr"/>
+      <c r="P113" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:50:00</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>11:50:00</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr"/>
+      <c r="E114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr"/>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr"/>
+      <c r="M114" s="2" t="inlineStr"/>
+      <c r="N114" s="2" t="inlineStr"/>
+      <c r="O114" s="2" t="inlineStr"/>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 11:55:00</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>11:55:00</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr"/>
+      <c r="E115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr"/>
+      <c r="G115" s="2" t="inlineStr"/>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr"/>
+      <c r="K115" s="2" t="inlineStr"/>
+      <c r="L115" s="2" t="inlineStr"/>
+      <c r="M115" s="2" t="inlineStr"/>
+      <c r="N115" s="2" t="inlineStr"/>
+      <c r="O115" s="2" t="inlineStr"/>
+      <c r="P115" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:20:00</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>12:20:00</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr"/>
+      <c r="E116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="2" t="inlineStr"/>
+      <c r="M116" s="2" t="inlineStr"/>
+      <c r="N116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr"/>
+      <c r="P116" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:25:00</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>12:25:00</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr"/>
+      <c r="E117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="2" t="inlineStr"/>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr"/>
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr"/>
+      <c r="M117" s="2" t="inlineStr"/>
+      <c r="N117" s="2" t="inlineStr"/>
+      <c r="O117" s="2" t="inlineStr"/>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:30:00</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr"/>
+      <c r="E118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr"/>
+      <c r="G118" s="2" t="inlineStr"/>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr"/>
+      <c r="N118" s="2" t="inlineStr"/>
+      <c r="O118" s="2" t="inlineStr"/>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:35:00</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>12:35:00</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>12:35</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr"/>
+      <c r="E119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr"/>
+      <c r="G119" s="2" t="inlineStr"/>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr"/>
+      <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr"/>
+      <c r="N119" s="2" t="inlineStr"/>
+      <c r="O119" s="2" t="inlineStr"/>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:40:00</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>12:40:00</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr"/>
+      <c r="E120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr"/>
+      <c r="G120" s="2" t="inlineStr"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr"/>
+      <c r="N120" s="2" t="inlineStr"/>
+      <c r="O120" s="2" t="inlineStr"/>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:45:00</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr"/>
+      <c r="E121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="inlineStr"/>
+      <c r="G121" s="2" t="inlineStr"/>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr"/>
+      <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr"/>
+      <c r="N121" s="2" t="inlineStr"/>
+      <c r="O121" s="2" t="inlineStr"/>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:50:00</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>12:50:00</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr"/>
+      <c r="E122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr"/>
+      <c r="G122" s="2" t="inlineStr"/>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr"/>
+      <c r="N122" s="2" t="inlineStr"/>
+      <c r="O122" s="2" t="inlineStr"/>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 12:55:00</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>12:55:00</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr"/>
+      <c r="E123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="inlineStr"/>
+      <c r="G123" s="2" t="inlineStr"/>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr"/>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr"/>
+      <c r="N123" s="2" t="inlineStr"/>
+      <c r="O123" s="2" t="inlineStr"/>
+      <c r="P123" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:20:00</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>13:20:00</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>13:20</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr"/>
+      <c r="E124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr"/>
+      <c r="G124" s="2" t="inlineStr"/>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr"/>
+      <c r="N124" s="2" t="inlineStr"/>
+      <c r="O124" s="2" t="inlineStr"/>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:25:00</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>13:25:00</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr"/>
+      <c r="E125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr"/>
+      <c r="G125" s="2" t="inlineStr"/>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr"/>
+      <c r="N125" s="2" t="inlineStr"/>
+      <c r="O125" s="2" t="inlineStr"/>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:30:00</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>13:30:00</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr"/>
+      <c r="E126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="inlineStr"/>
+      <c r="G126" s="2" t="inlineStr"/>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr"/>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr"/>
+      <c r="N126" s="2" t="inlineStr"/>
+      <c r="O126" s="2" t="inlineStr"/>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:35:00</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>13:35:00</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr"/>
+      <c r="E127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="inlineStr"/>
+      <c r="G127" s="2" t="inlineStr"/>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr"/>
+      <c r="N127" s="2" t="inlineStr"/>
+      <c r="O127" s="2" t="inlineStr"/>
+      <c r="P127" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:40:00</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>13:40:00</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr"/>
+      <c r="E128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr"/>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="inlineStr"/>
+      <c r="L128" s="2" t="inlineStr"/>
+      <c r="M128" s="2" t="inlineStr"/>
+      <c r="N128" s="2" t="inlineStr"/>
+      <c r="O128" s="2" t="inlineStr"/>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:45:00</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr"/>
+      <c r="E129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="inlineStr"/>
+      <c r="G129" s="2" t="inlineStr"/>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr"/>
+      <c r="K129" s="2" t="inlineStr"/>
+      <c r="L129" s="2" t="inlineStr"/>
+      <c r="M129" s="2" t="inlineStr"/>
+      <c r="N129" s="2" t="inlineStr"/>
+      <c r="O129" s="2" t="inlineStr"/>
+      <c r="P129" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:50:00</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>13:50:00</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr"/>
+      <c r="E130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="inlineStr"/>
+      <c r="G130" s="2" t="inlineStr"/>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr"/>
+      <c r="L130" s="2" t="inlineStr"/>
+      <c r="M130" s="2" t="inlineStr"/>
+      <c r="N130" s="2" t="inlineStr"/>
+      <c r="O130" s="2" t="inlineStr"/>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 13:55:00</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>13:55:00</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr"/>
+      <c r="E131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="inlineStr"/>
+      <c r="G131" s="2" t="inlineStr"/>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr"/>
+      <c r="K131" s="2" t="inlineStr"/>
+      <c r="L131" s="2" t="inlineStr"/>
+      <c r="M131" s="2" t="inlineStr"/>
+      <c r="N131" s="2" t="inlineStr"/>
+      <c r="O131" s="2" t="inlineStr"/>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:20:00</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr"/>
+      <c r="E132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr"/>
+      <c r="G132" s="2" t="inlineStr"/>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="inlineStr"/>
+      <c r="L132" s="2" t="inlineStr"/>
+      <c r="M132" s="2" t="inlineStr"/>
+      <c r="N132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr"/>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:25:00</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>14:25:00</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr"/>
+      <c r="E133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="inlineStr"/>
+      <c r="G133" s="2" t="inlineStr"/>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr"/>
+      <c r="K133" s="2" t="inlineStr"/>
+      <c r="L133" s="2" t="inlineStr"/>
+      <c r="M133" s="2" t="inlineStr"/>
+      <c r="N133" s="2" t="inlineStr"/>
+      <c r="O133" s="2" t="inlineStr"/>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:30:00</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>14:30:00</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr"/>
+      <c r="E134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr"/>
+      <c r="G134" s="2" t="inlineStr"/>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr"/>
+      <c r="L134" s="2" t="inlineStr"/>
+      <c r="M134" s="2" t="inlineStr"/>
+      <c r="N134" s="2" t="inlineStr"/>
+      <c r="O134" s="2" t="inlineStr"/>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:35:00</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>14:35:00</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr"/>
+      <c r="E135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="inlineStr"/>
+      <c r="G135" s="2" t="inlineStr"/>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr"/>
+      <c r="K135" s="2" t="inlineStr"/>
+      <c r="L135" s="2" t="inlineStr"/>
+      <c r="M135" s="2" t="inlineStr"/>
+      <c r="N135" s="2" t="inlineStr"/>
+      <c r="O135" s="2" t="inlineStr"/>
+      <c r="P135" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:40:00</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>14:40:00</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr"/>
+      <c r="E136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr"/>
+      <c r="G136" s="2" t="inlineStr"/>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr"/>
+      <c r="N136" s="2" t="inlineStr"/>
+      <c r="O136" s="2" t="inlineStr"/>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:45:00</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr"/>
+      <c r="E137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="inlineStr"/>
+      <c r="G137" s="2" t="inlineStr"/>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr"/>
+      <c r="K137" s="2" t="inlineStr"/>
+      <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr"/>
+      <c r="N137" s="2" t="inlineStr"/>
+      <c r="O137" s="2" t="inlineStr"/>
+      <c r="P137" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:50:00</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>14:50:00</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr"/>
+      <c r="E138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr"/>
+      <c r="G138" s="2" t="inlineStr"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr"/>
+      <c r="M138" s="2" t="inlineStr"/>
+      <c r="N138" s="2" t="inlineStr"/>
+      <c r="O138" s="2" t="inlineStr"/>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 14:55:00</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>14:55:00</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr"/>
+      <c r="E139" s="2" t="inlineStr"/>
+      <c r="F139" s="2" t="inlineStr"/>
+      <c r="G139" s="2" t="inlineStr"/>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr"/>
+      <c r="L139" s="2" t="inlineStr"/>
+      <c r="M139" s="2" t="inlineStr"/>
+      <c r="N139" s="2" t="inlineStr"/>
+      <c r="O139" s="2" t="inlineStr"/>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03 15:20:00</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>15:20:00</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>15:20</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr"/>
+      <c r="E140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr"/>
+      <c r="G140" s="2" t="inlineStr"/>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>✗ NO</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr"/>
+      <c r="M140" s="2" t="inlineStr"/>
+      <c r="N140" s="2" t="inlineStr"/>
+      <c r="O140" s="2" t="inlineStr"/>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>❌ Data not initialized</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>